<commit_message>
solved today Leetcode problem using Binary search
</commit_message>
<xml_diff>
--- a/DSA_shortcuts.xlsx
+++ b/DSA_shortcuts.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pdeepak\Documents\personal\Study\IP_Address\DSA\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD8BF91-C177-4CC8-BFEA-9FB10471C2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
   <si>
     <t>Topic</t>
   </si>
@@ -122,9 +128,6 @@
     <t>G1</t>
   </si>
   <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <b/>
@@ -266,9 +269,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <b/>
         <sz val="11"/>
@@ -345,9 +345,6 @@
     <t>G3</t>
   </si>
   <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <b/>
@@ -531,9 +528,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <b/>
         <sz val="11"/>
@@ -694,9 +688,6 @@
     <t>G5</t>
   </si>
   <si>
-    <r>
-      <t/>
-    </r>
     <r>
       <rPr>
         <b/>
@@ -776,9 +767,6 @@
   </si>
   <si>
     <r>
-      <t/>
-    </r>
-    <r>
       <rPr>
         <b/>
         <sz val="11"/>
@@ -1080,14 +1068,23 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>don't allocate vector&lt;int&gt;  unnecessarily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">don't use vector&lt;int&gt; for returning 2 values 
+--&gt; use pair&lt;int,int&gt; instead </t>
+  </si>
+  <si>
+    <t>Use const for function parameters if possible</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1107,6 +1104,21 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1136,41 +1148,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1181,10 +1193,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1222,71 +1234,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1314,7 +1326,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1337,11 +1349,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1350,13 +1362,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1366,7 +1378,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1375,7 +1387,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1384,7 +1396,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1392,10 +1404,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1460,21 +1472,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="6" width="6.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="30.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="52.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="6.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1484,14 +1496,17 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="I1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1501,14 +1516,17 @@
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
+      <c r="I2" s="7" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="2" t="s">
         <v>10</v>
@@ -1516,129 +1534,133 @@
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>9</v>
       </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="47.25">
+    <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="47.25">
+    <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="75">
+    <row r="6" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="75">
+    <row r="7" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="129.75">
+    <row r="8" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="116.25">
+    <row r="9" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="60.75">
+    <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;KFF8C00 CONFIDENTIAL&amp;1#_x000D_</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Leetcode DSA today - solved using bruteforce math
</commit_message>
<xml_diff>
--- a/DSA_shortcuts.xlsx
+++ b/DSA_shortcuts.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pdeepak\Documents\personal\Study\IP_Address\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD8BF91-C177-4CC8-BFEA-9FB10471C2AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEABC7C-C1ED-4D30-A7F4-8A8BCD02B69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
   <si>
     <t>Topic</t>
   </si>
@@ -1078,6 +1079,20 @@
   </si>
   <si>
     <t>Use const for function parameters if possible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">learn segment trees and try out the separate squares 2
+https://leetcode.com/problems/separate-squares-ii/?envType=daily-question&amp;envId=2026-01-14
+</t>
+  </si>
+  <si>
+    <t>n/m</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>m</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1144,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1144,11 +1159,238 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1171,6 +1413,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1483,7 +1745,7 @@
     <col min="2" max="2" width="30.88671875" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="52" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.21875" customWidth="1"/>
+    <col min="9" max="9" width="47.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -1544,7 +1806,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -1559,6 +1821,9 @@
       </c>
       <c r="E4" t="s">
         <v>9</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -1663,4 +1928,388 @@
     <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;KFF8C00 CONFIDENTIAL&amp;1#_x000D_</oddHeader>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB7018E7-9A20-4CB1-B8AA-78E813728157}">
+  <dimension ref="D2:AT29"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="8">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8">
+        <v>2</v>
+      </c>
+      <c r="G4" s="11">
+        <v>3</v>
+      </c>
+      <c r="H4" s="11">
+        <v>4</v>
+      </c>
+      <c r="I4" s="11">
+        <v>5</v>
+      </c>
+      <c r="J4" s="11">
+        <v>6</v>
+      </c>
+      <c r="K4" s="11">
+        <v>7</v>
+      </c>
+      <c r="L4" s="11">
+        <v>8</v>
+      </c>
+      <c r="M4" s="8">
+        <v>9</v>
+      </c>
+      <c r="N4" s="8">
+        <v>10</v>
+      </c>
+      <c r="O4" s="8">
+        <v>11</v>
+      </c>
+      <c r="P4" s="8">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>13</v>
+      </c>
+      <c r="R4" s="8">
+        <v>14</v>
+      </c>
+      <c r="S4" s="8">
+        <v>15</v>
+      </c>
+      <c r="T4" s="8">
+        <v>16</v>
+      </c>
+      <c r="U4" s="8">
+        <v>17</v>
+      </c>
+      <c r="V4" s="8">
+        <v>18</v>
+      </c>
+      <c r="W4" s="8">
+        <v>19</v>
+      </c>
+      <c r="X4" s="8">
+        <v>20</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>21</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>22</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>23</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>24</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>25</v>
+      </c>
+      <c r="AD4" s="8">
+        <v>26</v>
+      </c>
+      <c r="AE4" s="8">
+        <v>27</v>
+      </c>
+      <c r="AF4" s="8">
+        <v>28</v>
+      </c>
+      <c r="AG4" s="8">
+        <v>29</v>
+      </c>
+      <c r="AH4" s="8">
+        <v>30</v>
+      </c>
+      <c r="AI4" s="8">
+        <v>31</v>
+      </c>
+      <c r="AJ4" s="11">
+        <v>32</v>
+      </c>
+      <c r="AK4" s="11">
+        <v>33</v>
+      </c>
+      <c r="AL4" s="11">
+        <v>34</v>
+      </c>
+      <c r="AM4" s="11">
+        <v>35</v>
+      </c>
+      <c r="AN4" s="11">
+        <v>36</v>
+      </c>
+      <c r="AO4" s="8">
+        <v>37</v>
+      </c>
+      <c r="AP4" s="8">
+        <v>38</v>
+      </c>
+      <c r="AQ4" s="8">
+        <v>39</v>
+      </c>
+      <c r="AR4" s="8">
+        <v>40</v>
+      </c>
+      <c r="AS4" s="11">
+        <v>41</v>
+      </c>
+      <c r="AT4" s="11">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E5" s="8">
+        <v>2</v>
+      </c>
+      <c r="F5" s="13"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="26"/>
+      <c r="S5" s="14"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="14"/>
+      <c r="W5" s="26"/>
+      <c r="X5" s="26"/>
+      <c r="Y5" s="26"/>
+      <c r="Z5" s="26"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="14"/>
+      <c r="AC5" s="14"/>
+      <c r="AD5" s="26"/>
+      <c r="AE5" s="14"/>
+      <c r="AF5" s="12"/>
+      <c r="AG5" s="13"/>
+      <c r="AH5" s="12"/>
+      <c r="AI5" s="10"/>
+      <c r="AJ5" s="23"/>
+      <c r="AK5" s="9"/>
+      <c r="AL5" s="9"/>
+      <c r="AM5" s="15"/>
+      <c r="AN5" s="9"/>
+      <c r="AO5" s="12"/>
+      <c r="AP5" s="10"/>
+      <c r="AQ5" s="10"/>
+      <c r="AR5" s="13"/>
+      <c r="AS5" s="9"/>
+      <c r="AT5" s="24"/>
+    </row>
+    <row r="6" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E6" s="16">
+        <v>3</v>
+      </c>
+      <c r="F6" s="15"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="17"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="17"/>
+      <c r="X6" s="17"/>
+      <c r="Y6" s="17"/>
+      <c r="Z6" s="17"/>
+      <c r="AA6" s="15"/>
+      <c r="AB6" s="15"/>
+      <c r="AC6" s="15"/>
+      <c r="AD6" s="17"/>
+      <c r="AE6" s="15"/>
+      <c r="AF6" s="17"/>
+      <c r="AG6" s="15"/>
+      <c r="AH6" s="15"/>
+      <c r="AI6" s="15"/>
+      <c r="AJ6" s="15"/>
+      <c r="AK6" s="9"/>
+      <c r="AL6" s="9"/>
+      <c r="AM6" s="15"/>
+      <c r="AN6" s="9"/>
+      <c r="AO6" s="15"/>
+      <c r="AP6" s="15"/>
+      <c r="AQ6" s="17"/>
+      <c r="AR6" s="15"/>
+      <c r="AS6" s="9"/>
+      <c r="AT6" s="15"/>
+    </row>
+    <row r="7" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E7" s="16">
+        <v>4</v>
+      </c>
+      <c r="F7" s="15"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="17"/>
+      <c r="O7" s="17"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="17"/>
+      <c r="U7" s="17"/>
+      <c r="V7" s="15"/>
+      <c r="W7" s="17"/>
+      <c r="X7" s="17"/>
+      <c r="Y7" s="17"/>
+      <c r="Z7" s="17"/>
+      <c r="AA7" s="15"/>
+      <c r="AB7" s="15"/>
+      <c r="AC7" s="15"/>
+      <c r="AD7" s="17"/>
+      <c r="AE7" s="15"/>
+      <c r="AF7" s="17"/>
+      <c r="AG7" s="15"/>
+      <c r="AH7" s="15"/>
+      <c r="AI7" s="15"/>
+      <c r="AJ7" s="15"/>
+      <c r="AK7" s="9"/>
+      <c r="AL7" s="9"/>
+      <c r="AM7" s="15"/>
+      <c r="AN7" s="9"/>
+      <c r="AO7" s="15"/>
+      <c r="AP7" s="15"/>
+      <c r="AQ7" s="17"/>
+      <c r="AR7" s="15"/>
+      <c r="AS7" s="9"/>
+      <c r="AT7" s="15"/>
+    </row>
+    <row r="8" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E8" s="16">
+        <v>5</v>
+      </c>
+      <c r="F8" s="15"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="17"/>
+      <c r="O8" s="17"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="17"/>
+      <c r="S8" s="15"/>
+      <c r="T8" s="17"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="15"/>
+      <c r="W8" s="17"/>
+      <c r="X8" s="17"/>
+      <c r="Y8" s="17"/>
+      <c r="Z8" s="17"/>
+      <c r="AA8" s="15"/>
+      <c r="AB8" s="15"/>
+      <c r="AC8" s="15"/>
+      <c r="AD8" s="17"/>
+      <c r="AE8" s="15"/>
+      <c r="AF8" s="17"/>
+      <c r="AG8" s="15"/>
+      <c r="AH8" s="15"/>
+      <c r="AI8" s="15"/>
+      <c r="AJ8" s="15"/>
+      <c r="AK8" s="9"/>
+      <c r="AL8" s="9"/>
+      <c r="AM8" s="15"/>
+      <c r="AN8" s="9"/>
+      <c r="AO8" s="15"/>
+      <c r="AP8" s="15"/>
+      <c r="AQ8" s="17"/>
+      <c r="AR8" s="15"/>
+      <c r="AS8" s="9"/>
+      <c r="AT8" s="15"/>
+    </row>
+    <row r="9" spans="4:46" x14ac:dyDescent="0.3">
+      <c r="E9" s="8">
+        <v>6</v>
+      </c>
+      <c r="F9" s="18"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="27"/>
+      <c r="U9" s="27"/>
+      <c r="V9" s="22"/>
+      <c r="W9" s="27"/>
+      <c r="X9" s="27"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="20"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="22"/>
+      <c r="AC9" s="22"/>
+      <c r="AD9" s="27"/>
+      <c r="AE9" s="22"/>
+      <c r="AF9" s="19"/>
+      <c r="AG9" s="18"/>
+      <c r="AH9" s="19"/>
+      <c r="AI9" s="20"/>
+      <c r="AJ9" s="18"/>
+      <c r="AK9" s="21"/>
+      <c r="AL9" s="21"/>
+      <c r="AM9" s="22"/>
+      <c r="AN9" s="21"/>
+      <c r="AO9" s="19"/>
+      <c r="AP9" s="18"/>
+      <c r="AQ9" s="19"/>
+      <c r="AR9" s="18"/>
+      <c r="AS9" s="21"/>
+      <c r="AT9" s="22"/>
+    </row>
+    <row r="29" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J29" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
NodeJs learning - WebSockets
</commit_message>
<xml_diff>
--- a/DSA_shortcuts.xlsx
+++ b/DSA_shortcuts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pdeepak\Documents\personal\Study\IP_Address\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEABC7C-C1ED-4D30-A7F4-8A8BCD02B69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC1D8CC-5F9A-4DA6-A594-EFD0289A2835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1086,13 +1086,17 @@
 </t>
   </si>
   <si>
-    <t>n/m</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
-    <t>m</t>
+    <t>Algorithm</t>
+  </si>
+  <si>
+    <t>Majority voting algorithm</t>
+  </si>
+  <si>
+    <t>track count, start from count = 0, ele = nums[0]
+Now iterate,
+ele != nums[i] --&gt; count--
+else count++
+return ele after checking frequency</t>
   </si>
 </sst>
 </file>
@@ -1144,7 +1148,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1159,238 +1163,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1413,26 +1190,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1932,382 +1693,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB7018E7-9A20-4CB1-B8AA-78E813728157}">
-  <dimension ref="D2:AT29"/>
+  <dimension ref="A2:B3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.44140625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" style="8" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="8"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="F2" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="91.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="3" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="D4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="8">
-        <v>1</v>
-      </c>
-      <c r="F4" s="8">
-        <v>2</v>
-      </c>
-      <c r="G4" s="11">
-        <v>3</v>
-      </c>
-      <c r="H4" s="11">
-        <v>4</v>
-      </c>
-      <c r="I4" s="11">
-        <v>5</v>
-      </c>
-      <c r="J4" s="11">
-        <v>6</v>
-      </c>
-      <c r="K4" s="11">
-        <v>7</v>
-      </c>
-      <c r="L4" s="11">
-        <v>8</v>
-      </c>
-      <c r="M4" s="8">
-        <v>9</v>
-      </c>
-      <c r="N4" s="8">
-        <v>10</v>
-      </c>
-      <c r="O4" s="8">
-        <v>11</v>
-      </c>
-      <c r="P4" s="8">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="8">
-        <v>13</v>
-      </c>
-      <c r="R4" s="8">
-        <v>14</v>
-      </c>
-      <c r="S4" s="8">
-        <v>15</v>
-      </c>
-      <c r="T4" s="8">
-        <v>16</v>
-      </c>
-      <c r="U4" s="8">
-        <v>17</v>
-      </c>
-      <c r="V4" s="8">
-        <v>18</v>
-      </c>
-      <c r="W4" s="8">
-        <v>19</v>
-      </c>
-      <c r="X4" s="8">
-        <v>20</v>
-      </c>
-      <c r="Y4" s="8">
-        <v>21</v>
-      </c>
-      <c r="Z4" s="8">
-        <v>22</v>
-      </c>
-      <c r="AA4" s="8">
-        <v>23</v>
-      </c>
-      <c r="AB4" s="8">
-        <v>24</v>
-      </c>
-      <c r="AC4" s="8">
-        <v>25</v>
-      </c>
-      <c r="AD4" s="8">
-        <v>26</v>
-      </c>
-      <c r="AE4" s="8">
-        <v>27</v>
-      </c>
-      <c r="AF4" s="8">
-        <v>28</v>
-      </c>
-      <c r="AG4" s="8">
-        <v>29</v>
-      </c>
-      <c r="AH4" s="8">
-        <v>30</v>
-      </c>
-      <c r="AI4" s="8">
-        <v>31</v>
-      </c>
-      <c r="AJ4" s="11">
-        <v>32</v>
-      </c>
-      <c r="AK4" s="11">
-        <v>33</v>
-      </c>
-      <c r="AL4" s="11">
-        <v>34</v>
-      </c>
-      <c r="AM4" s="11">
-        <v>35</v>
-      </c>
-      <c r="AN4" s="11">
-        <v>36</v>
-      </c>
-      <c r="AO4" s="8">
-        <v>37</v>
-      </c>
-      <c r="AP4" s="8">
-        <v>38</v>
-      </c>
-      <c r="AQ4" s="8">
-        <v>39</v>
-      </c>
-      <c r="AR4" s="8">
-        <v>40</v>
-      </c>
-      <c r="AS4" s="11">
-        <v>41</v>
-      </c>
-      <c r="AT4" s="11">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E5" s="8">
-        <v>2</v>
-      </c>
-      <c r="F5" s="13"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="26"/>
-      <c r="U5" s="26"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="26"/>
-      <c r="X5" s="26"/>
-      <c r="Y5" s="26"/>
-      <c r="Z5" s="26"/>
-      <c r="AA5" s="14"/>
-      <c r="AB5" s="14"/>
-      <c r="AC5" s="14"/>
-      <c r="AD5" s="26"/>
-      <c r="AE5" s="14"/>
-      <c r="AF5" s="12"/>
-      <c r="AG5" s="13"/>
-      <c r="AH5" s="12"/>
-      <c r="AI5" s="10"/>
-      <c r="AJ5" s="23"/>
-      <c r="AK5" s="9"/>
-      <c r="AL5" s="9"/>
-      <c r="AM5" s="15"/>
-      <c r="AN5" s="9"/>
-      <c r="AO5" s="12"/>
-      <c r="AP5" s="10"/>
-      <c r="AQ5" s="10"/>
-      <c r="AR5" s="13"/>
-      <c r="AS5" s="9"/>
-      <c r="AT5" s="24"/>
-    </row>
-    <row r="6" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E6" s="16">
-        <v>3</v>
-      </c>
-      <c r="F6" s="15"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="17"/>
-      <c r="S6" s="15"/>
-      <c r="T6" s="17"/>
-      <c r="U6" s="17"/>
-      <c r="V6" s="15"/>
-      <c r="W6" s="17"/>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="17"/>
-      <c r="AA6" s="15"/>
-      <c r="AB6" s="15"/>
-      <c r="AC6" s="15"/>
-      <c r="AD6" s="17"/>
-      <c r="AE6" s="15"/>
-      <c r="AF6" s="17"/>
-      <c r="AG6" s="15"/>
-      <c r="AH6" s="15"/>
-      <c r="AI6" s="15"/>
-      <c r="AJ6" s="15"/>
-      <c r="AK6" s="9"/>
-      <c r="AL6" s="9"/>
-      <c r="AM6" s="15"/>
-      <c r="AN6" s="9"/>
-      <c r="AO6" s="15"/>
-      <c r="AP6" s="15"/>
-      <c r="AQ6" s="17"/>
-      <c r="AR6" s="15"/>
-      <c r="AS6" s="9"/>
-      <c r="AT6" s="15"/>
-    </row>
-    <row r="7" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E7" s="16">
-        <v>4</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="15"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="17"/>
-      <c r="S7" s="15"/>
-      <c r="T7" s="17"/>
-      <c r="U7" s="17"/>
-      <c r="V7" s="15"/>
-      <c r="W7" s="17"/>
-      <c r="X7" s="17"/>
-      <c r="Y7" s="17"/>
-      <c r="Z7" s="17"/>
-      <c r="AA7" s="15"/>
-      <c r="AB7" s="15"/>
-      <c r="AC7" s="15"/>
-      <c r="AD7" s="17"/>
-      <c r="AE7" s="15"/>
-      <c r="AF7" s="17"/>
-      <c r="AG7" s="15"/>
-      <c r="AH7" s="15"/>
-      <c r="AI7" s="15"/>
-      <c r="AJ7" s="15"/>
-      <c r="AK7" s="9"/>
-      <c r="AL7" s="9"/>
-      <c r="AM7" s="15"/>
-      <c r="AN7" s="9"/>
-      <c r="AO7" s="15"/>
-      <c r="AP7" s="15"/>
-      <c r="AQ7" s="17"/>
-      <c r="AR7" s="15"/>
-      <c r="AS7" s="9"/>
-      <c r="AT7" s="15"/>
-    </row>
-    <row r="8" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E8" s="16">
-        <v>5</v>
-      </c>
-      <c r="F8" s="15"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="17"/>
-      <c r="S8" s="15"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="17"/>
-      <c r="V8" s="15"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="17"/>
-      <c r="Y8" s="17"/>
-      <c r="Z8" s="17"/>
-      <c r="AA8" s="15"/>
-      <c r="AB8" s="15"/>
-      <c r="AC8" s="15"/>
-      <c r="AD8" s="17"/>
-      <c r="AE8" s="15"/>
-      <c r="AF8" s="17"/>
-      <c r="AG8" s="15"/>
-      <c r="AH8" s="15"/>
-      <c r="AI8" s="15"/>
-      <c r="AJ8" s="15"/>
-      <c r="AK8" s="9"/>
-      <c r="AL8" s="9"/>
-      <c r="AM8" s="15"/>
-      <c r="AN8" s="9"/>
-      <c r="AO8" s="15"/>
-      <c r="AP8" s="15"/>
-      <c r="AQ8" s="17"/>
-      <c r="AR8" s="15"/>
-      <c r="AS8" s="9"/>
-      <c r="AT8" s="15"/>
-    </row>
-    <row r="9" spans="4:46" x14ac:dyDescent="0.3">
-      <c r="E9" s="8">
-        <v>6</v>
-      </c>
-      <c r="F9" s="18"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="19"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="19"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="19"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="27"/>
-      <c r="U9" s="27"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="27"/>
-      <c r="X9" s="27"/>
-      <c r="Y9" s="19"/>
-      <c r="Z9" s="20"/>
-      <c r="AA9" s="18"/>
-      <c r="AB9" s="22"/>
-      <c r="AC9" s="22"/>
-      <c r="AD9" s="27"/>
-      <c r="AE9" s="22"/>
-      <c r="AF9" s="19"/>
-      <c r="AG9" s="18"/>
-      <c r="AH9" s="19"/>
-      <c r="AI9" s="20"/>
-      <c r="AJ9" s="18"/>
-      <c r="AK9" s="21"/>
-      <c r="AL9" s="21"/>
-      <c r="AM9" s="22"/>
-      <c r="AN9" s="21"/>
-      <c r="AO9" s="19"/>
-      <c r="AP9" s="18"/>
-      <c r="AQ9" s="19"/>
-      <c r="AR9" s="18"/>
-      <c r="AS9" s="21"/>
-      <c r="AT9" s="22"/>
-    </row>
-    <row r="29" spans="10:10" x14ac:dyDescent="0.3">
-      <c r="J29" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>